<commit_message>
Update Data and Code
</commit_message>
<xml_diff>
--- a/data/city_crosswalk.xlsx
+++ b/data/city_crosswalk.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28227"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28324"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Robert\OneDrive\Desktop\Bobby\GitHub\Skyscrapers\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CECB1E94-1689-41B3-B5C7-BCF6B56F34C9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{243FD9A1-E007-4BEF-A24C-78E26E4FC117}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{96C4E9D1-39CB-4160-B661-174130F89492}"/>
   </bookViews>
@@ -17,7 +17,7 @@
     <sheet name="Crosswalk" sheetId="2" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">Crosswalk!$A$1:$C$773</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">Crosswalk!$A$1:$C$782</definedName>
     <definedName name="IQ_CH">110000</definedName>
     <definedName name="IQ_CQ">5000</definedName>
     <definedName name="IQ_CY">10000</definedName>
@@ -70,7 +70,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2424" uniqueCount="1638">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2442" uniqueCount="1648">
   <si>
     <t>name_city</t>
   </si>
@@ -7084,6 +7084,36 @@
   </si>
   <si>
     <t>Pearl River Delta</t>
+  </si>
+  <si>
+    <t>Nacka</t>
+  </si>
+  <si>
+    <t>Sigtuna</t>
+  </si>
+  <si>
+    <t>Sollentuna</t>
+  </si>
+  <si>
+    <t>Taby</t>
+  </si>
+  <si>
+    <t>Upplands Vasby</t>
+  </si>
+  <si>
+    <t>Stanford</t>
+  </si>
+  <si>
+    <t>San Francisco Bay Area</t>
+  </si>
+  <si>
+    <t>Osan</t>
+  </si>
+  <si>
+    <t>Pyeongtaek</t>
+  </si>
+  <si>
+    <t>Yeoju</t>
   </si>
 </sst>
 </file>
@@ -21381,6 +21411,99 @@
     </row>
   </sheetData>
   <mergeCells count="105">
+    <mergeCell ref="A947:D947"/>
+    <mergeCell ref="A952:D952"/>
+    <mergeCell ref="A966:D966"/>
+    <mergeCell ref="A896:D896"/>
+    <mergeCell ref="A903:D903"/>
+    <mergeCell ref="A912:D912"/>
+    <mergeCell ref="A922:D922"/>
+    <mergeCell ref="A926:D926"/>
+    <mergeCell ref="A930:D930"/>
+    <mergeCell ref="A843:D843"/>
+    <mergeCell ref="A866:D866"/>
+    <mergeCell ref="A871:D871"/>
+    <mergeCell ref="A878:D878"/>
+    <mergeCell ref="A884:D884"/>
+    <mergeCell ref="A888:D888"/>
+    <mergeCell ref="A777:D777"/>
+    <mergeCell ref="A795:D795"/>
+    <mergeCell ref="A799:D799"/>
+    <mergeCell ref="A808:D808"/>
+    <mergeCell ref="A835:D835"/>
+    <mergeCell ref="A839:D839"/>
+    <mergeCell ref="A740:D740"/>
+    <mergeCell ref="A744:D744"/>
+    <mergeCell ref="A748:D748"/>
+    <mergeCell ref="A752:D752"/>
+    <mergeCell ref="A756:D756"/>
+    <mergeCell ref="A769:D769"/>
+    <mergeCell ref="A710:D710"/>
+    <mergeCell ref="A714:D714"/>
+    <mergeCell ref="A718:D718"/>
+    <mergeCell ref="A726:D726"/>
+    <mergeCell ref="A730:D730"/>
+    <mergeCell ref="A736:D736"/>
+    <mergeCell ref="A617:D617"/>
+    <mergeCell ref="A625:D625"/>
+    <mergeCell ref="A629:D629"/>
+    <mergeCell ref="A683:D683"/>
+    <mergeCell ref="A695:D695"/>
+    <mergeCell ref="A702:D702"/>
+    <mergeCell ref="A561:D561"/>
+    <mergeCell ref="A566:D566"/>
+    <mergeCell ref="A570:D570"/>
+    <mergeCell ref="A601:D601"/>
+    <mergeCell ref="A605:D605"/>
+    <mergeCell ref="A612:D612"/>
+    <mergeCell ref="A514:D514"/>
+    <mergeCell ref="A518:D518"/>
+    <mergeCell ref="A525:D525"/>
+    <mergeCell ref="A531:D531"/>
+    <mergeCell ref="A552:D552"/>
+    <mergeCell ref="A556:D556"/>
+    <mergeCell ref="A446:D446"/>
+    <mergeCell ref="A451:D451"/>
+    <mergeCell ref="A466:D466"/>
+    <mergeCell ref="A470:D470"/>
+    <mergeCell ref="A478:D478"/>
+    <mergeCell ref="A493:D493"/>
+    <mergeCell ref="A394:D394"/>
+    <mergeCell ref="A399:D399"/>
+    <mergeCell ref="A404:D404"/>
+    <mergeCell ref="A410:D410"/>
+    <mergeCell ref="A416:D416"/>
+    <mergeCell ref="A442:D442"/>
+    <mergeCell ref="A347:D347"/>
+    <mergeCell ref="A360:D360"/>
+    <mergeCell ref="A366:D366"/>
+    <mergeCell ref="A373:D373"/>
+    <mergeCell ref="A378:D378"/>
+    <mergeCell ref="A382:D382"/>
+    <mergeCell ref="A310:D310"/>
+    <mergeCell ref="A314:D314"/>
+    <mergeCell ref="A327:D327"/>
+    <mergeCell ref="A332:D332"/>
+    <mergeCell ref="A338:D338"/>
+    <mergeCell ref="A342:D342"/>
+    <mergeCell ref="A262:D262"/>
+    <mergeCell ref="A266:D266"/>
+    <mergeCell ref="A271:D271"/>
+    <mergeCell ref="A275:D275"/>
+    <mergeCell ref="A286:D286"/>
+    <mergeCell ref="A290:D290"/>
+    <mergeCell ref="A202:D202"/>
+    <mergeCell ref="A211:D211"/>
+    <mergeCell ref="A223:D223"/>
+    <mergeCell ref="A236:D236"/>
+    <mergeCell ref="A240:D240"/>
+    <mergeCell ref="A253:D253"/>
+    <mergeCell ref="A103:D103"/>
+    <mergeCell ref="A110:D110"/>
+    <mergeCell ref="A175:D175"/>
+    <mergeCell ref="A182:D182"/>
+    <mergeCell ref="A186:D186"/>
+    <mergeCell ref="A198:D198"/>
     <mergeCell ref="A54:D54"/>
     <mergeCell ref="A61:D61"/>
     <mergeCell ref="A68:D68"/>
@@ -21393,99 +21516,6 @@
     <mergeCell ref="A15:D15"/>
     <mergeCell ref="A45:D45"/>
     <mergeCell ref="A49:D49"/>
-    <mergeCell ref="A202:D202"/>
-    <mergeCell ref="A211:D211"/>
-    <mergeCell ref="A223:D223"/>
-    <mergeCell ref="A236:D236"/>
-    <mergeCell ref="A240:D240"/>
-    <mergeCell ref="A253:D253"/>
-    <mergeCell ref="A103:D103"/>
-    <mergeCell ref="A110:D110"/>
-    <mergeCell ref="A175:D175"/>
-    <mergeCell ref="A182:D182"/>
-    <mergeCell ref="A186:D186"/>
-    <mergeCell ref="A198:D198"/>
-    <mergeCell ref="A310:D310"/>
-    <mergeCell ref="A314:D314"/>
-    <mergeCell ref="A327:D327"/>
-    <mergeCell ref="A332:D332"/>
-    <mergeCell ref="A338:D338"/>
-    <mergeCell ref="A342:D342"/>
-    <mergeCell ref="A262:D262"/>
-    <mergeCell ref="A266:D266"/>
-    <mergeCell ref="A271:D271"/>
-    <mergeCell ref="A275:D275"/>
-    <mergeCell ref="A286:D286"/>
-    <mergeCell ref="A290:D290"/>
-    <mergeCell ref="A394:D394"/>
-    <mergeCell ref="A399:D399"/>
-    <mergeCell ref="A404:D404"/>
-    <mergeCell ref="A410:D410"/>
-    <mergeCell ref="A416:D416"/>
-    <mergeCell ref="A442:D442"/>
-    <mergeCell ref="A347:D347"/>
-    <mergeCell ref="A360:D360"/>
-    <mergeCell ref="A366:D366"/>
-    <mergeCell ref="A373:D373"/>
-    <mergeCell ref="A378:D378"/>
-    <mergeCell ref="A382:D382"/>
-    <mergeCell ref="A514:D514"/>
-    <mergeCell ref="A518:D518"/>
-    <mergeCell ref="A525:D525"/>
-    <mergeCell ref="A531:D531"/>
-    <mergeCell ref="A552:D552"/>
-    <mergeCell ref="A556:D556"/>
-    <mergeCell ref="A446:D446"/>
-    <mergeCell ref="A451:D451"/>
-    <mergeCell ref="A466:D466"/>
-    <mergeCell ref="A470:D470"/>
-    <mergeCell ref="A478:D478"/>
-    <mergeCell ref="A493:D493"/>
-    <mergeCell ref="A617:D617"/>
-    <mergeCell ref="A625:D625"/>
-    <mergeCell ref="A629:D629"/>
-    <mergeCell ref="A683:D683"/>
-    <mergeCell ref="A695:D695"/>
-    <mergeCell ref="A702:D702"/>
-    <mergeCell ref="A561:D561"/>
-    <mergeCell ref="A566:D566"/>
-    <mergeCell ref="A570:D570"/>
-    <mergeCell ref="A601:D601"/>
-    <mergeCell ref="A605:D605"/>
-    <mergeCell ref="A612:D612"/>
-    <mergeCell ref="A740:D740"/>
-    <mergeCell ref="A744:D744"/>
-    <mergeCell ref="A748:D748"/>
-    <mergeCell ref="A752:D752"/>
-    <mergeCell ref="A756:D756"/>
-    <mergeCell ref="A769:D769"/>
-    <mergeCell ref="A710:D710"/>
-    <mergeCell ref="A714:D714"/>
-    <mergeCell ref="A718:D718"/>
-    <mergeCell ref="A726:D726"/>
-    <mergeCell ref="A730:D730"/>
-    <mergeCell ref="A736:D736"/>
-    <mergeCell ref="A843:D843"/>
-    <mergeCell ref="A866:D866"/>
-    <mergeCell ref="A871:D871"/>
-    <mergeCell ref="A878:D878"/>
-    <mergeCell ref="A884:D884"/>
-    <mergeCell ref="A888:D888"/>
-    <mergeCell ref="A777:D777"/>
-    <mergeCell ref="A795:D795"/>
-    <mergeCell ref="A799:D799"/>
-    <mergeCell ref="A808:D808"/>
-    <mergeCell ref="A835:D835"/>
-    <mergeCell ref="A839:D839"/>
-    <mergeCell ref="A947:D947"/>
-    <mergeCell ref="A952:D952"/>
-    <mergeCell ref="A966:D966"/>
-    <mergeCell ref="A896:D896"/>
-    <mergeCell ref="A903:D903"/>
-    <mergeCell ref="A912:D912"/>
-    <mergeCell ref="A922:D922"/>
-    <mergeCell ref="A926:D926"/>
-    <mergeCell ref="A930:D930"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink ref="A2" r:id="rId1" display="https://skyscraperpage.com/cities/?cityID=149" xr:uid="{DD369ABA-25BD-4D20-89A5-33EC39EDAA77}"/>
@@ -23396,7 +23426,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{38210FFA-F41E-4694-9E11-07D3D8230991}">
-  <dimension ref="A1:C773"/>
+  <dimension ref="A1:C782"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="29.6640625" bestFit="1" customWidth="1"/>
@@ -29227,8 +29257,8 @@
       <c r="A530" t="s">
         <v>1603</v>
       </c>
-      <c r="B530" t="e">
-        <v>#N/A</v>
+      <c r="B530">
+        <v>3560</v>
       </c>
       <c r="C530" t="s">
         <v>1131</v>
@@ -29238,8 +29268,8 @@
       <c r="A531" t="s">
         <v>1130</v>
       </c>
-      <c r="B531" t="e">
-        <v>#N/A</v>
+      <c r="B531">
+        <v>1447</v>
       </c>
       <c r="C531" t="s">
         <v>1131</v>
@@ -29249,8 +29279,8 @@
       <c r="A532" t="s">
         <v>1131</v>
       </c>
-      <c r="B532" t="e">
-        <v>#N/A</v>
+      <c r="B532">
+        <v>326</v>
       </c>
       <c r="C532" t="s">
         <v>1131</v>
@@ -29282,8 +29312,8 @@
       <c r="A535" t="s">
         <v>1132</v>
       </c>
-      <c r="B535" t="e">
-        <v>#N/A</v>
+      <c r="B535">
+        <v>165</v>
       </c>
       <c r="C535" t="s">
         <v>1133</v>
@@ -29293,8 +29323,8 @@
       <c r="A536" t="s">
         <v>1133</v>
       </c>
-      <c r="B536" t="e">
-        <v>#N/A</v>
+      <c r="B536">
+        <v>164</v>
       </c>
       <c r="C536" t="s">
         <v>1133</v>
@@ -29304,8 +29334,8 @@
       <c r="A537" t="s">
         <v>1134</v>
       </c>
-      <c r="B537" t="e">
-        <v>#N/A</v>
+      <c r="B537">
+        <v>3157</v>
       </c>
       <c r="C537" t="s">
         <v>1133</v>
@@ -29315,8 +29345,8 @@
       <c r="A538" t="s">
         <v>1135</v>
       </c>
-      <c r="B538" t="e">
-        <v>#N/A</v>
+      <c r="B538">
+        <v>2821</v>
       </c>
       <c r="C538" t="s">
         <v>1133</v>
@@ -29326,8 +29356,8 @@
       <c r="A539" t="s">
         <v>1136</v>
       </c>
-      <c r="B539" t="e">
-        <v>#N/A</v>
+      <c r="B539">
+        <v>6133</v>
       </c>
       <c r="C539" t="s">
         <v>1137</v>
@@ -29337,8 +29367,8 @@
       <c r="A540" t="s">
         <v>1137</v>
       </c>
-      <c r="B540" t="e">
-        <v>#N/A</v>
+      <c r="B540">
+        <v>327</v>
       </c>
       <c r="C540" t="s">
         <v>1137</v>
@@ -29425,8 +29455,8 @@
       <c r="A548" t="s">
         <v>1138</v>
       </c>
-      <c r="B548" t="e">
-        <v>#N/A</v>
+      <c r="B548">
+        <v>6879</v>
       </c>
       <c r="C548" t="s">
         <v>1139</v>
@@ -29436,8 +29466,8 @@
       <c r="A549" t="s">
         <v>1139</v>
       </c>
-      <c r="B549" t="e">
-        <v>#N/A</v>
+      <c r="B549">
+        <v>1378</v>
       </c>
       <c r="C549" t="s">
         <v>1139</v>
@@ -29447,8 +29477,8 @@
       <c r="A550" t="s">
         <v>1140</v>
       </c>
-      <c r="B550" t="e">
-        <v>#N/A</v>
+      <c r="B550">
+        <v>7655</v>
       </c>
       <c r="C550" t="s">
         <v>1139</v>
@@ -29458,8 +29488,8 @@
       <c r="A551" t="s">
         <v>1607</v>
       </c>
-      <c r="B551" t="e">
-        <v>#N/A</v>
+      <c r="B551">
+        <v>4255</v>
       </c>
       <c r="C551" t="s">
         <v>1139</v>
@@ -29469,8 +29499,8 @@
       <c r="A552" t="s">
         <v>1608</v>
       </c>
-      <c r="B552" t="e">
-        <v>#N/A</v>
+      <c r="B552">
+        <v>3615</v>
       </c>
       <c r="C552" t="s">
         <v>1139</v>
@@ -29480,8 +29510,8 @@
       <c r="A553" t="s">
         <v>1141</v>
       </c>
-      <c r="B553" t="e">
-        <v>#N/A</v>
+      <c r="B553">
+        <v>3600</v>
       </c>
       <c r="C553" t="s">
         <v>1142</v>
@@ -29491,8 +29521,8 @@
       <c r="A554" t="s">
         <v>1142</v>
       </c>
-      <c r="B554" t="e">
-        <v>#N/A</v>
+      <c r="B554">
+        <v>2098</v>
       </c>
       <c r="C554" t="s">
         <v>1142</v>
@@ -29502,8 +29532,8 @@
       <c r="A555" t="s">
         <v>1143</v>
       </c>
-      <c r="B555" t="e">
-        <v>#N/A</v>
+      <c r="B555">
+        <v>7933</v>
       </c>
       <c r="C555" t="s">
         <v>1145</v>
@@ -29513,8 +29543,8 @@
       <c r="A556" t="s">
         <v>1144</v>
       </c>
-      <c r="B556" t="e">
-        <v>#N/A</v>
+      <c r="B556">
+        <v>6473</v>
       </c>
       <c r="C556" t="s">
         <v>1145</v>
@@ -29524,8 +29554,8 @@
       <c r="A557" t="s">
         <v>1145</v>
       </c>
-      <c r="B557" t="e">
-        <v>#N/A</v>
+      <c r="B557">
+        <v>65</v>
       </c>
       <c r="C557" t="s">
         <v>1145</v>
@@ -29535,8 +29565,8 @@
       <c r="A558" t="s">
         <v>1146</v>
       </c>
-      <c r="B558" t="e">
-        <v>#N/A</v>
+      <c r="B558">
+        <v>8105</v>
       </c>
       <c r="C558" t="s">
         <v>1145</v>
@@ -29546,8 +29576,8 @@
       <c r="A559" t="s">
         <v>1609</v>
       </c>
-      <c r="B559" t="e">
-        <v>#N/A</v>
+      <c r="B559">
+        <v>2454</v>
       </c>
       <c r="C559" t="s">
         <v>1147</v>
@@ -29557,8 +29587,8 @@
       <c r="A560" t="s">
         <v>1147</v>
       </c>
-      <c r="B560" t="e">
-        <v>#N/A</v>
+      <c r="B560">
+        <v>2453</v>
       </c>
       <c r="C560" t="s">
         <v>1147</v>
@@ -29568,8 +29598,8 @@
       <c r="A561" t="s">
         <v>1148</v>
       </c>
-      <c r="B561" t="e">
-        <v>#N/A</v>
+      <c r="B561">
+        <v>3362</v>
       </c>
       <c r="C561" t="s">
         <v>1148</v>
@@ -29579,8 +29609,8 @@
       <c r="A562" t="s">
         <v>1149</v>
       </c>
-      <c r="B562" t="e">
-        <v>#N/A</v>
+      <c r="B562">
+        <v>7656</v>
       </c>
       <c r="C562" t="s">
         <v>1148</v>
@@ -29590,8 +29620,8 @@
       <c r="A563" t="s">
         <v>1150</v>
       </c>
-      <c r="B563" t="e">
-        <v>#N/A</v>
+      <c r="B563">
+        <v>162</v>
       </c>
       <c r="C563" t="s">
         <v>1150</v>
@@ -29601,8 +29631,8 @@
       <c r="A564" t="s">
         <v>1151</v>
       </c>
-      <c r="B564" t="e">
-        <v>#N/A</v>
+      <c r="B564">
+        <v>4237</v>
       </c>
       <c r="C564" t="s">
         <v>1150</v>
@@ -29612,8 +29642,8 @@
       <c r="A565" t="s">
         <v>1152</v>
       </c>
-      <c r="B565" t="e">
-        <v>#N/A</v>
+      <c r="B565">
+        <v>1211</v>
       </c>
       <c r="C565" t="s">
         <v>1153</v>
@@ -29623,8 +29653,8 @@
       <c r="A566" t="s">
         <v>1153</v>
       </c>
-      <c r="B566" t="e">
-        <v>#N/A</v>
+      <c r="B566">
+        <v>893</v>
       </c>
       <c r="C566" t="s">
         <v>1153</v>
@@ -29634,8 +29664,8 @@
       <c r="A567" t="s">
         <v>1154</v>
       </c>
-      <c r="B567" t="e">
-        <v>#N/A</v>
+      <c r="B567">
+        <v>3901</v>
       </c>
       <c r="C567" t="s">
         <v>1155</v>
@@ -29645,8 +29675,8 @@
       <c r="A568" t="s">
         <v>1155</v>
       </c>
-      <c r="B568" t="e">
-        <v>#N/A</v>
+      <c r="B568">
+        <v>3390</v>
       </c>
       <c r="C568" t="s">
         <v>1155</v>
@@ -29678,8 +29708,8 @@
       <c r="A571" t="s">
         <v>1158</v>
       </c>
-      <c r="B571" t="e">
-        <v>#N/A</v>
+      <c r="B571">
+        <v>1908</v>
       </c>
       <c r="C571" t="s">
         <v>1162</v>
@@ -29689,8 +29719,8 @@
       <c r="A572" t="s">
         <v>1159</v>
       </c>
-      <c r="B572" t="e">
-        <v>#N/A</v>
+      <c r="B572">
+        <v>2609</v>
       </c>
       <c r="C572" t="s">
         <v>1162</v>
@@ -29700,8 +29730,8 @@
       <c r="A573" t="s">
         <v>1160</v>
       </c>
-      <c r="B573" t="e">
-        <v>#N/A</v>
+      <c r="B573">
+        <v>1087</v>
       </c>
       <c r="C573" t="s">
         <v>1162</v>
@@ -29711,8 +29741,8 @@
       <c r="A574" t="s">
         <v>1161</v>
       </c>
-      <c r="B574" t="e">
-        <v>#N/A</v>
+      <c r="B574">
+        <v>1691</v>
       </c>
       <c r="C574" t="s">
         <v>1162</v>
@@ -29722,8 +29752,8 @@
       <c r="A575" t="s">
         <v>1162</v>
       </c>
-      <c r="B575" t="e">
-        <v>#N/A</v>
+      <c r="B575">
+        <v>897</v>
       </c>
       <c r="C575" t="s">
         <v>1162</v>
@@ -29733,8 +29763,8 @@
       <c r="A576" t="s">
         <v>1163</v>
       </c>
-      <c r="B576" t="e">
-        <v>#N/A</v>
+      <c r="B576">
+        <v>2373</v>
       </c>
       <c r="C576" t="s">
         <v>1162</v>
@@ -29744,8 +29774,8 @@
       <c r="A577" t="s">
         <v>1164</v>
       </c>
-      <c r="B577" t="e">
-        <v>#N/A</v>
+      <c r="B577">
+        <v>1102</v>
       </c>
       <c r="C577" t="s">
         <v>1162</v>
@@ -29755,8 +29785,8 @@
       <c r="A578" t="s">
         <v>1165</v>
       </c>
-      <c r="B578" t="e">
-        <v>#N/A</v>
+      <c r="B578">
+        <v>3610</v>
       </c>
       <c r="C578" t="s">
         <v>1162</v>
@@ -29766,8 +29796,8 @@
       <c r="A579" t="s">
         <v>1610</v>
       </c>
-      <c r="B579" t="e">
-        <v>#N/A</v>
+      <c r="B579">
+        <v>3436</v>
       </c>
       <c r="C579" t="s">
         <v>1162</v>
@@ -29788,8 +29818,8 @@
       <c r="A581" t="s">
         <v>1166</v>
       </c>
-      <c r="B581" t="e">
-        <v>#N/A</v>
+      <c r="B581">
+        <v>397</v>
       </c>
       <c r="C581" t="s">
         <v>1168</v>
@@ -29799,8 +29829,8 @@
       <c r="A582" t="s">
         <v>1167</v>
       </c>
-      <c r="B582" t="e">
-        <v>#N/A</v>
+      <c r="B582">
+        <v>91</v>
       </c>
       <c r="C582" t="s">
         <v>1168</v>
@@ -29810,8 +29840,8 @@
       <c r="A583" t="s">
         <v>1168</v>
       </c>
-      <c r="B583" t="e">
-        <v>#N/A</v>
+      <c r="B583">
+        <v>90</v>
       </c>
       <c r="C583" t="s">
         <v>1168</v>
@@ -29821,8 +29851,8 @@
       <c r="A584" t="s">
         <v>1612</v>
       </c>
-      <c r="B584" t="e">
-        <v>#N/A</v>
+      <c r="B584">
+        <v>6941</v>
       </c>
       <c r="C584" t="s">
         <v>1168</v>
@@ -29832,8 +29862,8 @@
       <c r="A585" t="s">
         <v>1613</v>
       </c>
-      <c r="B585" t="e">
-        <v>#N/A</v>
+      <c r="B585">
+        <v>391</v>
       </c>
       <c r="C585" t="s">
         <v>1168</v>
@@ -29847,7 +29877,7 @@
         <v>209</v>
       </c>
       <c r="C586" t="s">
-        <v>1176</v>
+        <v>1644</v>
       </c>
     </row>
     <row r="587" spans="1:3" x14ac:dyDescent="0.3">
@@ -29858,7 +29888,7 @@
         <v>5029</v>
       </c>
       <c r="C587" t="s">
-        <v>1176</v>
+        <v>1644</v>
       </c>
     </row>
     <row r="588" spans="1:3" x14ac:dyDescent="0.3">
@@ -29869,169 +29899,169 @@
         <v>6055</v>
       </c>
       <c r="C588" t="s">
-        <v>1176</v>
+        <v>1644</v>
       </c>
     </row>
     <row r="589" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A589" t="s">
         <v>1172</v>
       </c>
-      <c r="B589" t="e">
-        <v>#N/A</v>
+      <c r="B589">
+        <v>5025</v>
       </c>
       <c r="C589" t="s">
-        <v>1176</v>
+        <v>1644</v>
       </c>
     </row>
     <row r="590" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A590" t="s">
         <v>1614</v>
       </c>
-      <c r="B590" t="e">
-        <v>#N/A</v>
+      <c r="B590">
+        <v>6058</v>
       </c>
       <c r="C590" t="s">
-        <v>1176</v>
+        <v>1644</v>
       </c>
     </row>
     <row r="591" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A591" t="s">
         <v>1173</v>
       </c>
-      <c r="B591" t="e">
-        <v>#N/A</v>
+      <c r="B591">
+        <v>5018</v>
       </c>
       <c r="C591" t="s">
-        <v>1176</v>
+        <v>1644</v>
       </c>
     </row>
     <row r="592" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A592" t="s">
         <v>1174</v>
       </c>
-      <c r="B592" t="e">
-        <v>#N/A</v>
+      <c r="B592">
+        <v>113</v>
       </c>
       <c r="C592" t="s">
-        <v>1176</v>
+        <v>1644</v>
       </c>
     </row>
     <row r="593" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A593" t="s">
         <v>1175</v>
       </c>
-      <c r="B593" t="e">
-        <v>#N/A</v>
+      <c r="B593">
+        <v>3836</v>
       </c>
       <c r="C593" t="s">
-        <v>1176</v>
+        <v>1644</v>
       </c>
     </row>
     <row r="594" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A594" t="s">
         <v>897</v>
       </c>
-      <c r="B594" t="e">
-        <v>#N/A</v>
+      <c r="B594">
+        <v>128</v>
       </c>
       <c r="C594" t="s">
-        <v>1176</v>
+        <v>1644</v>
       </c>
     </row>
     <row r="595" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A595" t="s">
         <v>1176</v>
       </c>
-      <c r="B595" t="e">
-        <v>#N/A</v>
+      <c r="B595">
+        <v>114</v>
       </c>
       <c r="C595" t="s">
-        <v>1176</v>
+        <v>1644</v>
       </c>
     </row>
     <row r="596" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A596" t="s">
         <v>1177</v>
       </c>
-      <c r="B596" t="e">
-        <v>#N/A</v>
+      <c r="B596">
+        <v>123</v>
       </c>
       <c r="C596" t="s">
-        <v>1176</v>
+        <v>1644</v>
       </c>
     </row>
     <row r="597" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A597" t="s">
         <v>1178</v>
       </c>
-      <c r="B597" t="e">
-        <v>#N/A</v>
+      <c r="B597">
+        <v>5017</v>
       </c>
       <c r="C597" t="s">
-        <v>1176</v>
+        <v>1644</v>
       </c>
     </row>
     <row r="598" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A598" t="s">
         <v>1179</v>
       </c>
-      <c r="B598" t="e">
-        <v>#N/A</v>
+      <c r="B598">
+        <v>3414</v>
       </c>
       <c r="C598" t="s">
-        <v>1176</v>
+        <v>1644</v>
       </c>
     </row>
     <row r="599" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A599" t="s">
         <v>1180</v>
       </c>
-      <c r="B599" t="e">
-        <v>#N/A</v>
+      <c r="B599">
+        <v>5014</v>
       </c>
       <c r="C599" t="s">
-        <v>1176</v>
+        <v>1644</v>
       </c>
     </row>
     <row r="600" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A600" t="s">
-        <v>1181</v>
-      </c>
-      <c r="B600" t="e">
-        <v>#N/A</v>
+        <v>1643</v>
+      </c>
+      <c r="B600">
+        <v>124</v>
       </c>
       <c r="C600" t="s">
-        <v>1176</v>
+        <v>1644</v>
       </c>
     </row>
     <row r="601" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A601" t="s">
-        <v>1182</v>
-      </c>
-      <c r="B601" t="e">
-        <v>#N/A</v>
+        <v>1181</v>
+      </c>
+      <c r="B601">
+        <v>215</v>
       </c>
       <c r="C601" t="s">
-        <v>1176</v>
+        <v>1644</v>
       </c>
     </row>
     <row r="602" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A602" t="s">
-        <v>1183</v>
+        <v>1182</v>
       </c>
       <c r="B602">
-        <v>2224</v>
+        <v>220</v>
       </c>
       <c r="C602" t="s">
-        <v>1184</v>
+        <v>1644</v>
       </c>
     </row>
     <row r="603" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A603" t="s">
-        <v>1184</v>
-      </c>
-      <c r="B603" t="e">
-        <v>#N/A</v>
+        <v>1183</v>
+      </c>
+      <c r="B603">
+        <v>2224</v>
       </c>
       <c r="C603" t="s">
         <v>1184</v>
@@ -30039,21 +30069,21 @@
     </row>
     <row r="604" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A604" t="s">
-        <v>1185</v>
+        <v>1184</v>
       </c>
       <c r="B604">
-        <v>83</v>
+        <v>909</v>
       </c>
       <c r="C604" t="s">
-        <v>1189</v>
+        <v>1184</v>
       </c>
     </row>
     <row r="605" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A605" t="s">
-        <v>1186</v>
-      </c>
-      <c r="B605" t="e">
-        <v>#N/A</v>
+        <v>1185</v>
+      </c>
+      <c r="B605">
+        <v>83</v>
       </c>
       <c r="C605" t="s">
         <v>1189</v>
@@ -30061,10 +30091,10 @@
     </row>
     <row r="606" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A606" t="s">
-        <v>1615</v>
-      </c>
-      <c r="B606" t="e">
-        <v>#N/A</v>
+        <v>1186</v>
+      </c>
+      <c r="B606">
+        <v>1331</v>
       </c>
       <c r="C606" t="s">
         <v>1189</v>
@@ -30072,10 +30102,10 @@
     </row>
     <row r="607" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A607" t="s">
-        <v>1187</v>
-      </c>
-      <c r="B607" t="e">
-        <v>#N/A</v>
+        <v>1615</v>
+      </c>
+      <c r="B607">
+        <v>1332</v>
       </c>
       <c r="C607" t="s">
         <v>1189</v>
@@ -30083,10 +30113,10 @@
     </row>
     <row r="608" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A608" t="s">
-        <v>1188</v>
-      </c>
-      <c r="B608" t="e">
-        <v>#N/A</v>
+        <v>1187</v>
+      </c>
+      <c r="B608">
+        <v>1327</v>
       </c>
       <c r="C608" t="s">
         <v>1189</v>
@@ -30094,10 +30124,10 @@
     </row>
     <row r="609" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A609" t="s">
-        <v>1189</v>
-      </c>
-      <c r="B609" t="e">
-        <v>#N/A</v>
+        <v>1188</v>
+      </c>
+      <c r="B609">
+        <v>406</v>
       </c>
       <c r="C609" t="s">
         <v>1189</v>
@@ -30105,10 +30135,10 @@
     </row>
     <row r="610" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A610" t="s">
-        <v>1190</v>
-      </c>
-      <c r="B610" t="e">
-        <v>#N/A</v>
+        <v>1189</v>
+      </c>
+      <c r="B610">
+        <v>27</v>
       </c>
       <c r="C610" t="s">
         <v>1189</v>
@@ -30116,21 +30146,21 @@
     </row>
     <row r="611" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A611" t="s">
-        <v>1191</v>
+        <v>1190</v>
       </c>
       <c r="B611">
-        <v>7503</v>
+        <v>79</v>
       </c>
       <c r="C611" t="s">
-        <v>1209</v>
+        <v>1189</v>
       </c>
     </row>
     <row r="612" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A612" t="s">
-        <v>1192</v>
+        <v>1191</v>
       </c>
       <c r="B612">
-        <v>8737</v>
+        <v>7503</v>
       </c>
       <c r="C612" t="s">
         <v>1209</v>
@@ -30138,10 +30168,10 @@
     </row>
     <row r="613" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A613" t="s">
-        <v>1193</v>
+        <v>1192</v>
       </c>
       <c r="B613">
-        <v>2833</v>
+        <v>8737</v>
       </c>
       <c r="C613" t="s">
         <v>1209</v>
@@ -30149,10 +30179,10 @@
     </row>
     <row r="614" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A614" t="s">
-        <v>1194</v>
+        <v>1193</v>
       </c>
       <c r="B614">
-        <v>2836</v>
+        <v>2833</v>
       </c>
       <c r="C614" t="s">
         <v>1209</v>
@@ -30160,10 +30190,10 @@
     </row>
     <row r="615" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A615" t="s">
-        <v>1195</v>
+        <v>1194</v>
       </c>
       <c r="B615">
-        <v>1749</v>
+        <v>2836</v>
       </c>
       <c r="C615" t="s">
         <v>1209</v>
@@ -30171,10 +30201,10 @@
     </row>
     <row r="616" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A616" t="s">
-        <v>1196</v>
-      </c>
-      <c r="B616" t="e">
-        <v>#N/A</v>
+        <v>1195</v>
+      </c>
+      <c r="B616">
+        <v>1749</v>
       </c>
       <c r="C616" t="s">
         <v>1209</v>
@@ -30182,10 +30212,10 @@
     </row>
     <row r="617" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A617" t="s">
-        <v>1197</v>
-      </c>
-      <c r="B617" t="e">
-        <v>#N/A</v>
+        <v>1196</v>
+      </c>
+      <c r="B617">
+        <v>7505</v>
       </c>
       <c r="C617" t="s">
         <v>1209</v>
@@ -30193,10 +30223,10 @@
     </row>
     <row r="618" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A618" t="s">
-        <v>1198</v>
-      </c>
-      <c r="B618" t="e">
-        <v>#N/A</v>
+        <v>1197</v>
+      </c>
+      <c r="B618">
+        <v>1759</v>
       </c>
       <c r="C618" t="s">
         <v>1209</v>
@@ -30204,10 +30234,10 @@
     </row>
     <row r="619" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A619" t="s">
-        <v>1199</v>
-      </c>
-      <c r="B619" t="e">
-        <v>#N/A</v>
+        <v>1198</v>
+      </c>
+      <c r="B619">
+        <v>2834</v>
       </c>
       <c r="C619" t="s">
         <v>1209</v>
@@ -30215,10 +30245,10 @@
     </row>
     <row r="620" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A620" t="s">
-        <v>1200</v>
-      </c>
-      <c r="B620" t="e">
-        <v>#N/A</v>
+        <v>1199</v>
+      </c>
+      <c r="B620">
+        <v>7476</v>
       </c>
       <c r="C620" t="s">
         <v>1209</v>
@@ -30226,10 +30256,10 @@
     </row>
     <row r="621" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A621" t="s">
-        <v>1201</v>
-      </c>
-      <c r="B621" t="e">
-        <v>#N/A</v>
+        <v>1200</v>
+      </c>
+      <c r="B621">
+        <v>1765</v>
       </c>
       <c r="C621" t="s">
         <v>1209</v>
@@ -30237,10 +30267,10 @@
     </row>
     <row r="622" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A622" t="s">
-        <v>1202</v>
-      </c>
-      <c r="B622" t="e">
-        <v>#N/A</v>
+        <v>1201</v>
+      </c>
+      <c r="B622">
+        <v>7480</v>
       </c>
       <c r="C622" t="s">
         <v>1209</v>
@@ -30248,10 +30278,10 @@
     </row>
     <row r="623" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A623" t="s">
-        <v>1203</v>
-      </c>
-      <c r="B623" t="e">
-        <v>#N/A</v>
+        <v>1202</v>
+      </c>
+      <c r="B623">
+        <v>7481</v>
       </c>
       <c r="C623" t="s">
         <v>1209</v>
@@ -30259,10 +30289,10 @@
     </row>
     <row r="624" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A624" t="s">
-        <v>1204</v>
-      </c>
-      <c r="B624" t="e">
-        <v>#N/A</v>
+        <v>1203</v>
+      </c>
+      <c r="B624">
+        <v>5488</v>
       </c>
       <c r="C624" t="s">
         <v>1209</v>
@@ -30270,10 +30300,10 @@
     </row>
     <row r="625" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A625" t="s">
-        <v>1205</v>
-      </c>
-      <c r="B625" t="e">
-        <v>#N/A</v>
+        <v>1204</v>
+      </c>
+      <c r="B625">
+        <v>6646</v>
       </c>
       <c r="C625" t="s">
         <v>1209</v>
@@ -30281,10 +30311,10 @@
     </row>
     <row r="626" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A626" t="s">
-        <v>1206</v>
-      </c>
-      <c r="B626" t="e">
-        <v>#N/A</v>
+        <v>1205</v>
+      </c>
+      <c r="B626">
+        <v>1756</v>
       </c>
       <c r="C626" t="s">
         <v>1209</v>
@@ -30292,10 +30322,10 @@
     </row>
     <row r="627" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A627" t="s">
-        <v>1207</v>
-      </c>
-      <c r="B627" t="e">
-        <v>#N/A</v>
+        <v>1206</v>
+      </c>
+      <c r="B627">
+        <v>5511</v>
       </c>
       <c r="C627" t="s">
         <v>1209</v>
@@ -30303,10 +30333,10 @@
     </row>
     <row r="628" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A628" t="s">
-        <v>1208</v>
-      </c>
-      <c r="B628" t="e">
-        <v>#N/A</v>
+        <v>1645</v>
+      </c>
+      <c r="B628">
+        <v>7477</v>
       </c>
       <c r="C628" t="s">
         <v>1209</v>
@@ -30314,10 +30344,10 @@
     </row>
     <row r="629" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A629" t="s">
-        <v>1209</v>
-      </c>
-      <c r="B629" t="e">
-        <v>#N/A</v>
+        <v>1207</v>
+      </c>
+      <c r="B629">
+        <v>7478</v>
       </c>
       <c r="C629" t="s">
         <v>1209</v>
@@ -30325,10 +30355,10 @@
     </row>
     <row r="630" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A630" t="s">
-        <v>1210</v>
-      </c>
-      <c r="B630" t="e">
-        <v>#N/A</v>
+        <v>1646</v>
+      </c>
+      <c r="B630">
+        <v>7479</v>
       </c>
       <c r="C630" t="s">
         <v>1209</v>
@@ -30336,10 +30366,10 @@
     </row>
     <row r="631" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A631" t="s">
-        <v>1211</v>
-      </c>
-      <c r="B631" t="e">
-        <v>#N/A</v>
+        <v>1208</v>
+      </c>
+      <c r="B631">
+        <v>1751</v>
       </c>
       <c r="C631" t="s">
         <v>1209</v>
@@ -30347,10 +30377,10 @@
     </row>
     <row r="632" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A632" t="s">
-        <v>1212</v>
-      </c>
-      <c r="B632" t="e">
-        <v>#N/A</v>
+        <v>1209</v>
+      </c>
+      <c r="B632">
+        <v>914</v>
       </c>
       <c r="C632" t="s">
         <v>1209</v>
@@ -30358,10 +30388,10 @@
     </row>
     <row r="633" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A633" t="s">
-        <v>1213</v>
-      </c>
-      <c r="B633" t="e">
-        <v>#N/A</v>
+        <v>1210</v>
+      </c>
+      <c r="B633">
+        <v>7504</v>
       </c>
       <c r="C633" t="s">
         <v>1209</v>
@@ -30369,10 +30399,10 @@
     </row>
     <row r="634" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A634" t="s">
-        <v>1214</v>
-      </c>
-      <c r="B634" t="e">
-        <v>#N/A</v>
+        <v>1211</v>
+      </c>
+      <c r="B634">
+        <v>1755</v>
       </c>
       <c r="C634" t="s">
         <v>1209</v>
@@ -30380,10 +30410,10 @@
     </row>
     <row r="635" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A635" t="s">
-        <v>1215</v>
-      </c>
-      <c r="B635" t="e">
-        <v>#N/A</v>
+        <v>1212</v>
+      </c>
+      <c r="B635">
+        <v>7475</v>
       </c>
       <c r="C635" t="s">
         <v>1209</v>
@@ -30391,98 +30421,98 @@
     </row>
     <row r="636" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A636" t="s">
-        <v>1216</v>
-      </c>
-      <c r="B636" t="e">
-        <v>#N/A</v>
+        <v>1213</v>
+      </c>
+      <c r="B636">
+        <v>7785</v>
       </c>
       <c r="C636" t="s">
-        <v>1217</v>
+        <v>1209</v>
       </c>
     </row>
     <row r="637" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A637" t="s">
-        <v>1217</v>
-      </c>
-      <c r="B637" t="e">
-        <v>#N/A</v>
+        <v>1214</v>
+      </c>
+      <c r="B637">
+        <v>7786</v>
       </c>
       <c r="C637" t="s">
-        <v>1217</v>
+        <v>1209</v>
       </c>
     </row>
     <row r="638" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A638" t="s">
-        <v>1218</v>
-      </c>
-      <c r="B638" t="e">
-        <v>#N/A</v>
+        <v>1647</v>
+      </c>
+      <c r="B638">
+        <v>7545</v>
       </c>
       <c r="C638" t="s">
-        <v>1219</v>
+        <v>1209</v>
       </c>
     </row>
     <row r="639" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A639" t="s">
-        <v>1219</v>
-      </c>
-      <c r="B639" t="e">
-        <v>#N/A</v>
+        <v>1215</v>
+      </c>
+      <c r="B639">
+        <v>7482</v>
       </c>
       <c r="C639" t="s">
-        <v>1219</v>
+        <v>1209</v>
       </c>
     </row>
     <row r="640" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A640" t="s">
-        <v>1118</v>
+        <v>1216</v>
       </c>
       <c r="B640">
-        <v>1415</v>
+        <v>7004</v>
       </c>
       <c r="C640" t="s">
-        <v>1637</v>
+        <v>1217</v>
       </c>
     </row>
     <row r="641" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A641" t="s">
-        <v>1119</v>
+        <v>1217</v>
       </c>
       <c r="B641">
-        <v>1416</v>
+        <v>6</v>
       </c>
       <c r="C641" t="s">
-        <v>1637</v>
+        <v>1217</v>
       </c>
     </row>
     <row r="642" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A642" t="s">
-        <v>1120</v>
+        <v>1218</v>
       </c>
       <c r="B642">
-        <v>25</v>
+        <v>1851</v>
       </c>
       <c r="C642" t="s">
-        <v>1637</v>
+        <v>1219</v>
       </c>
     </row>
     <row r="643" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A643" t="s">
-        <v>1121</v>
+        <v>1219</v>
       </c>
       <c r="B643">
-        <v>7</v>
+        <v>918</v>
       </c>
       <c r="C643" t="s">
-        <v>1637</v>
+        <v>1219</v>
       </c>
     </row>
     <row r="644" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A644" t="s">
-        <v>1122</v>
+        <v>1118</v>
       </c>
       <c r="B644">
-        <v>1641</v>
+        <v>1415</v>
       </c>
       <c r="C644" t="s">
         <v>1637</v>
@@ -30490,10 +30520,10 @@
     </row>
     <row r="645" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A645" t="s">
-        <v>1123</v>
+        <v>1119</v>
       </c>
       <c r="B645">
-        <v>1637</v>
+        <v>1416</v>
       </c>
       <c r="C645" t="s">
         <v>1637</v>
@@ -30501,10 +30531,10 @@
     </row>
     <row r="646" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A646" t="s">
-        <v>1124</v>
+        <v>1120</v>
       </c>
       <c r="B646">
-        <v>814</v>
+        <v>25</v>
       </c>
       <c r="C646" t="s">
         <v>1637</v>
@@ -30512,10 +30542,10 @@
     </row>
     <row r="647" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A647" t="s">
-        <v>1125</v>
+        <v>1121</v>
       </c>
       <c r="B647">
-        <v>24</v>
+        <v>7</v>
       </c>
       <c r="C647" t="s">
         <v>1637</v>
@@ -30523,10 +30553,10 @@
     </row>
     <row r="648" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A648" t="s">
-        <v>1126</v>
+        <v>1122</v>
       </c>
       <c r="B648">
-        <v>1636</v>
+        <v>1641</v>
       </c>
       <c r="C648" t="s">
         <v>1637</v>
@@ -30534,10 +30564,10 @@
     </row>
     <row r="649" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A649" t="s">
-        <v>1127</v>
+        <v>1123</v>
       </c>
       <c r="B649">
-        <v>1409</v>
+        <v>1637</v>
       </c>
       <c r="C649" t="s">
         <v>1637</v>
@@ -30545,54 +30575,54 @@
     </row>
     <row r="650" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A650" t="s">
-        <v>1220</v>
+        <v>1124</v>
       </c>
       <c r="B650">
-        <v>1497</v>
+        <v>814</v>
       </c>
       <c r="C650" t="s">
-        <v>1234</v>
+        <v>1637</v>
       </c>
     </row>
     <row r="651" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A651" t="s">
-        <v>1169</v>
+        <v>1125</v>
       </c>
       <c r="B651">
-        <v>1498</v>
+        <v>24</v>
       </c>
       <c r="C651" t="s">
-        <v>1234</v>
+        <v>1637</v>
       </c>
     </row>
     <row r="652" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A652" t="s">
-        <v>1221</v>
+        <v>1126</v>
       </c>
       <c r="B652">
-        <v>4866</v>
+        <v>1636</v>
       </c>
       <c r="C652" t="s">
-        <v>1234</v>
+        <v>1637</v>
       </c>
     </row>
     <row r="653" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A653" t="s">
-        <v>1222</v>
+        <v>1127</v>
       </c>
       <c r="B653">
-        <v>4865</v>
+        <v>1409</v>
       </c>
       <c r="C653" t="s">
-        <v>1234</v>
+        <v>1637</v>
       </c>
     </row>
     <row r="654" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A654" t="s">
-        <v>1223</v>
+        <v>1220</v>
       </c>
       <c r="B654">
-        <v>1499</v>
+        <v>1497</v>
       </c>
       <c r="C654" t="s">
         <v>1234</v>
@@ -30600,10 +30630,10 @@
     </row>
     <row r="655" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A655" t="s">
-        <v>1224</v>
+        <v>1169</v>
       </c>
       <c r="B655">
-        <v>484</v>
+        <v>1498</v>
       </c>
       <c r="C655" t="s">
         <v>1234</v>
@@ -30611,10 +30641,10 @@
     </row>
     <row r="656" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A656" t="s">
-        <v>1225</v>
-      </c>
-      <c r="B656" t="e">
-        <v>#N/A</v>
+        <v>1221</v>
+      </c>
+      <c r="B656">
+        <v>4866</v>
       </c>
       <c r="C656" t="s">
         <v>1234</v>
@@ -30622,10 +30652,10 @@
     </row>
     <row r="657" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A657" t="s">
-        <v>1226</v>
-      </c>
-      <c r="B657" t="e">
-        <v>#N/A</v>
+        <v>1222</v>
+      </c>
+      <c r="B657">
+        <v>4865</v>
       </c>
       <c r="C657" t="s">
         <v>1234</v>
@@ -30633,10 +30663,10 @@
     </row>
     <row r="658" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A658" t="s">
-        <v>1227</v>
-      </c>
-      <c r="B658" t="e">
-        <v>#N/A</v>
+        <v>1223</v>
+      </c>
+      <c r="B658">
+        <v>1499</v>
       </c>
       <c r="C658" t="s">
         <v>1234</v>
@@ -30644,10 +30674,10 @@
     </row>
     <row r="659" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A659" t="s">
-        <v>1616</v>
-      </c>
-      <c r="B659" t="e">
-        <v>#N/A</v>
+        <v>1224</v>
+      </c>
+      <c r="B659">
+        <v>484</v>
       </c>
       <c r="C659" t="s">
         <v>1234</v>
@@ -30655,10 +30685,10 @@
     </row>
     <row r="660" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A660" t="s">
-        <v>1228</v>
-      </c>
-      <c r="B660" t="e">
-        <v>#N/A</v>
+        <v>1225</v>
+      </c>
+      <c r="B660">
+        <v>4864</v>
       </c>
       <c r="C660" t="s">
         <v>1234</v>
@@ -30666,10 +30696,10 @@
     </row>
     <row r="661" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A661" t="s">
-        <v>1229</v>
-      </c>
-      <c r="B661" t="e">
-        <v>#N/A</v>
+        <v>1226</v>
+      </c>
+      <c r="B661">
+        <v>4863</v>
       </c>
       <c r="C661" t="s">
         <v>1234</v>
@@ -30677,10 +30707,10 @@
     </row>
     <row r="662" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A662" t="s">
-        <v>1617</v>
-      </c>
-      <c r="B662" t="e">
-        <v>#N/A</v>
+        <v>1227</v>
+      </c>
+      <c r="B662">
+        <v>1500</v>
       </c>
       <c r="C662" t="s">
         <v>1234</v>
@@ -30688,10 +30718,10 @@
     </row>
     <row r="663" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A663" t="s">
-        <v>1230</v>
-      </c>
-      <c r="B663" t="e">
-        <v>#N/A</v>
+        <v>1616</v>
+      </c>
+      <c r="B663">
+        <v>502</v>
       </c>
       <c r="C663" t="s">
         <v>1234</v>
@@ -30699,10 +30729,10 @@
     </row>
     <row r="664" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A664" t="s">
-        <v>1618</v>
-      </c>
-      <c r="B664" t="e">
-        <v>#N/A</v>
+        <v>1228</v>
+      </c>
+      <c r="B664">
+        <v>1501</v>
       </c>
       <c r="C664" t="s">
         <v>1234</v>
@@ -30710,10 +30740,10 @@
     </row>
     <row r="665" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A665" t="s">
-        <v>1231</v>
-      </c>
-      <c r="B665" t="e">
-        <v>#N/A</v>
+        <v>1229</v>
+      </c>
+      <c r="B665">
+        <v>6061</v>
       </c>
       <c r="C665" t="s">
         <v>1234</v>
@@ -30721,10 +30751,10 @@
     </row>
     <row r="666" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A666" t="s">
-        <v>1232</v>
-      </c>
-      <c r="B666" t="e">
-        <v>#N/A</v>
+        <v>1617</v>
+      </c>
+      <c r="B666">
+        <v>490</v>
       </c>
       <c r="C666" t="s">
         <v>1234</v>
@@ -30732,10 +30762,10 @@
     </row>
     <row r="667" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A667" t="s">
-        <v>1233</v>
-      </c>
-      <c r="B667" t="e">
-        <v>#N/A</v>
+        <v>1230</v>
+      </c>
+      <c r="B667">
+        <v>508</v>
       </c>
       <c r="C667" t="s">
         <v>1234</v>
@@ -30743,10 +30773,10 @@
     </row>
     <row r="668" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A668" t="s">
-        <v>1234</v>
-      </c>
-      <c r="B668" t="e">
-        <v>#N/A</v>
+        <v>1618</v>
+      </c>
+      <c r="B668">
+        <v>512</v>
       </c>
       <c r="C668" t="s">
         <v>1234</v>
@@ -30754,10 +30784,10 @@
     </row>
     <row r="669" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A669" t="s">
-        <v>1619</v>
-      </c>
-      <c r="B669" t="e">
-        <v>#N/A</v>
+        <v>1231</v>
+      </c>
+      <c r="B669">
+        <v>516</v>
       </c>
       <c r="C669" t="s">
         <v>1234</v>
@@ -30765,10 +30795,10 @@
     </row>
     <row r="670" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A670" t="s">
-        <v>1235</v>
-      </c>
-      <c r="B670" t="e">
-        <v>#N/A</v>
+        <v>1232</v>
+      </c>
+      <c r="B670">
+        <v>1502</v>
       </c>
       <c r="C670" t="s">
         <v>1234</v>
@@ -30776,461 +30806,461 @@
     </row>
     <row r="671" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A671" t="s">
-        <v>1236</v>
-      </c>
-      <c r="B671" t="e">
-        <v>#N/A</v>
+        <v>1233</v>
+      </c>
+      <c r="B671">
+        <v>4856</v>
       </c>
       <c r="C671" t="s">
-        <v>1238</v>
+        <v>1234</v>
       </c>
     </row>
     <row r="672" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A672" t="s">
-        <v>1237</v>
-      </c>
-      <c r="B672" t="e">
-        <v>#N/A</v>
+        <v>1234</v>
+      </c>
+      <c r="B672">
+        <v>518</v>
       </c>
       <c r="C672" t="s">
-        <v>1238</v>
+        <v>1234</v>
       </c>
     </row>
     <row r="673" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A673" t="s">
-        <v>1238</v>
-      </c>
-      <c r="B673" t="e">
-        <v>#N/A</v>
+        <v>1619</v>
+      </c>
+      <c r="B673">
+        <v>7050</v>
       </c>
       <c r="C673" t="s">
-        <v>1238</v>
+        <v>1234</v>
       </c>
     </row>
     <row r="674" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A674" t="s">
-        <v>1239</v>
-      </c>
-      <c r="B674" t="e">
-        <v>#N/A</v>
+        <v>1235</v>
+      </c>
+      <c r="B674">
+        <v>1503</v>
       </c>
       <c r="C674" t="s">
-        <v>1242</v>
+        <v>1234</v>
       </c>
     </row>
     <row r="675" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A675" t="s">
-        <v>1240</v>
-      </c>
-      <c r="B675" t="e">
-        <v>#N/A</v>
+        <v>1236</v>
+      </c>
+      <c r="B675">
+        <v>2402</v>
       </c>
       <c r="C675" t="s">
-        <v>1242</v>
+        <v>1238</v>
       </c>
     </row>
     <row r="676" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A676" t="s">
-        <v>1241</v>
-      </c>
-      <c r="B676" t="e">
-        <v>#N/A</v>
+        <v>1237</v>
+      </c>
+      <c r="B676">
+        <v>2051</v>
       </c>
       <c r="C676" t="s">
-        <v>1242</v>
+        <v>1238</v>
       </c>
     </row>
     <row r="677" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A677" t="s">
-        <v>1242</v>
-      </c>
-      <c r="B677" t="e">
-        <v>#N/A</v>
+        <v>1238</v>
+      </c>
+      <c r="B677">
+        <v>929</v>
       </c>
       <c r="C677" t="s">
-        <v>1242</v>
+        <v>1238</v>
       </c>
     </row>
     <row r="678" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A678" t="s">
-        <v>1243</v>
-      </c>
-      <c r="B678" t="e">
-        <v>#N/A</v>
+        <v>1638</v>
+      </c>
+      <c r="B678">
+        <v>2123</v>
       </c>
       <c r="C678" t="s">
-        <v>1242</v>
+        <v>1238</v>
       </c>
     </row>
     <row r="679" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A679" t="s">
-        <v>1244</v>
-      </c>
-      <c r="B679" t="e">
-        <v>#N/A</v>
+        <v>1639</v>
+      </c>
+      <c r="B679">
+        <v>2199</v>
       </c>
       <c r="C679" t="s">
-        <v>1246</v>
+        <v>1238</v>
       </c>
     </row>
     <row r="680" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A680" t="s">
-        <v>1245</v>
-      </c>
-      <c r="B680" t="e">
-        <v>#N/A</v>
+        <v>1640</v>
+      </c>
+      <c r="B680">
+        <v>2229</v>
       </c>
       <c r="C680" t="s">
-        <v>1246</v>
+        <v>1238</v>
       </c>
     </row>
     <row r="681" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A681" t="s">
-        <v>1246</v>
-      </c>
-      <c r="B681" t="e">
-        <v>#N/A</v>
+        <v>1641</v>
+      </c>
+      <c r="B681">
+        <v>2294</v>
       </c>
       <c r="C681" t="s">
-        <v>1246</v>
+        <v>1238</v>
       </c>
     </row>
     <row r="682" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A682" t="s">
-        <v>1247</v>
-      </c>
-      <c r="B682" t="e">
-        <v>#N/A</v>
+        <v>1642</v>
+      </c>
+      <c r="B682">
+        <v>1979</v>
       </c>
       <c r="C682" t="s">
-        <v>1246</v>
+        <v>1238</v>
       </c>
     </row>
     <row r="683" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A683" t="s">
-        <v>1248</v>
-      </c>
-      <c r="B683" t="e">
-        <v>#N/A</v>
+        <v>1239</v>
+      </c>
+      <c r="B683">
+        <v>2556</v>
       </c>
       <c r="C683" t="s">
-        <v>1249</v>
+        <v>1242</v>
       </c>
     </row>
     <row r="684" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A684" t="s">
-        <v>1249</v>
-      </c>
-      <c r="B684" t="e">
-        <v>#N/A</v>
+        <v>1240</v>
+      </c>
+      <c r="B684">
+        <v>2553</v>
       </c>
       <c r="C684" t="s">
-        <v>1249</v>
+        <v>1242</v>
       </c>
     </row>
     <row r="685" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A685" t="s">
-        <v>1250</v>
+        <v>1241</v>
       </c>
       <c r="B685">
-        <v>140</v>
+        <v>2554</v>
       </c>
       <c r="C685" t="s">
-        <v>1254</v>
+        <v>1242</v>
       </c>
     </row>
     <row r="686" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A686" t="s">
-        <v>1251</v>
-      </c>
-      <c r="B686" t="e">
-        <v>#N/A</v>
+        <v>1242</v>
+      </c>
+      <c r="B686">
+        <v>172</v>
       </c>
       <c r="C686" t="s">
-        <v>1254</v>
+        <v>1242</v>
       </c>
     </row>
     <row r="687" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A687" t="s">
-        <v>1252</v>
-      </c>
-      <c r="B687" t="e">
-        <v>#N/A</v>
+        <v>1243</v>
+      </c>
+      <c r="B687">
+        <v>2555</v>
       </c>
       <c r="C687" t="s">
-        <v>1254</v>
+        <v>1242</v>
       </c>
     </row>
     <row r="688" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A688" t="s">
-        <v>1253</v>
-      </c>
-      <c r="B688" t="e">
-        <v>#N/A</v>
+        <v>1244</v>
+      </c>
+      <c r="B688">
+        <v>765</v>
       </c>
       <c r="C688" t="s">
-        <v>1254</v>
+        <v>1246</v>
       </c>
     </row>
     <row r="689" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A689" t="s">
-        <v>1254</v>
-      </c>
-      <c r="B689" t="e">
-        <v>#N/A</v>
+        <v>1245</v>
+      </c>
+      <c r="B689">
+        <v>7594</v>
       </c>
       <c r="C689" t="s">
-        <v>1254</v>
+        <v>1246</v>
       </c>
     </row>
     <row r="690" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A690" t="s">
-        <v>1255</v>
-      </c>
-      <c r="B690" t="e">
-        <v>#N/A</v>
+        <v>1246</v>
+      </c>
+      <c r="B690">
+        <v>9</v>
       </c>
       <c r="C690" t="s">
-        <v>1254</v>
+        <v>1246</v>
       </c>
     </row>
     <row r="691" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A691" t="s">
-        <v>1256</v>
+        <v>1247</v>
       </c>
       <c r="B691">
-        <v>3100</v>
+        <v>942</v>
       </c>
       <c r="C691" t="s">
-        <v>1260</v>
+        <v>1246</v>
       </c>
     </row>
     <row r="692" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A692" t="s">
-        <v>1257</v>
+        <v>1248</v>
       </c>
       <c r="B692">
-        <v>6539</v>
+        <v>2055</v>
       </c>
       <c r="C692" t="s">
-        <v>1260</v>
+        <v>1249</v>
       </c>
     </row>
     <row r="693" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A693" t="s">
-        <v>1258</v>
+        <v>1249</v>
       </c>
       <c r="B693">
-        <v>709</v>
+        <v>941</v>
       </c>
       <c r="C693" t="s">
-        <v>1260</v>
+        <v>1249</v>
       </c>
     </row>
     <row r="694" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A694" t="s">
-        <v>1259</v>
+        <v>1250</v>
       </c>
       <c r="B694">
-        <v>886</v>
+        <v>140</v>
       </c>
       <c r="C694" t="s">
-        <v>1260</v>
+        <v>1254</v>
       </c>
     </row>
     <row r="695" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A695" t="s">
-        <v>1260</v>
+        <v>1251</v>
       </c>
       <c r="B695">
-        <v>948</v>
+        <v>5639</v>
       </c>
       <c r="C695" t="s">
-        <v>1260</v>
+        <v>1254</v>
       </c>
     </row>
     <row r="696" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A696" t="s">
-        <v>1261</v>
+        <v>1252</v>
       </c>
       <c r="B696">
-        <v>1053</v>
+        <v>5640</v>
       </c>
       <c r="C696" t="s">
-        <v>1265</v>
+        <v>1254</v>
       </c>
     </row>
     <row r="697" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A697" t="s">
-        <v>1262</v>
+        <v>1253</v>
       </c>
       <c r="B697">
-        <v>1086</v>
+        <v>419</v>
       </c>
       <c r="C697" t="s">
-        <v>1265</v>
+        <v>1254</v>
       </c>
     </row>
     <row r="698" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A698" t="s">
-        <v>1263</v>
+        <v>1254</v>
       </c>
       <c r="B698">
-        <v>5574</v>
+        <v>138</v>
       </c>
       <c r="C698" t="s">
-        <v>1265</v>
+        <v>1254</v>
       </c>
     </row>
     <row r="699" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A699" t="s">
-        <v>1264</v>
+        <v>1255</v>
       </c>
       <c r="B699">
-        <v>892</v>
+        <v>5641</v>
       </c>
       <c r="C699" t="s">
-        <v>1265</v>
+        <v>1254</v>
       </c>
     </row>
     <row r="700" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A700" t="s">
-        <v>1265</v>
+        <v>1256</v>
       </c>
       <c r="B700">
-        <v>952</v>
+        <v>3100</v>
       </c>
       <c r="C700" t="s">
-        <v>1265</v>
+        <v>1260</v>
       </c>
     </row>
     <row r="701" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A701" t="s">
-        <v>1266</v>
+        <v>1257</v>
       </c>
       <c r="B701">
-        <v>3575</v>
+        <v>6539</v>
       </c>
       <c r="C701" t="s">
-        <v>1265</v>
+        <v>1260</v>
       </c>
     </row>
     <row r="702" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A702" t="s">
-        <v>1267</v>
+        <v>1258</v>
       </c>
       <c r="B702">
-        <v>1018</v>
+        <v>709</v>
       </c>
       <c r="C702" t="s">
-        <v>1265</v>
+        <v>1260</v>
       </c>
     </row>
     <row r="703" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A703" t="s">
-        <v>1560</v>
+        <v>1259</v>
       </c>
       <c r="B703">
-        <v>8026</v>
+        <v>886</v>
       </c>
       <c r="C703" t="s">
-        <v>876</v>
+        <v>1260</v>
       </c>
     </row>
     <row r="704" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A704" t="s">
-        <v>870</v>
+        <v>1260</v>
       </c>
       <c r="B704">
-        <v>2495</v>
+        <v>948</v>
       </c>
       <c r="C704" t="s">
-        <v>876</v>
+        <v>1260</v>
       </c>
     </row>
     <row r="705" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A705" t="s">
-        <v>871</v>
+        <v>1261</v>
       </c>
       <c r="B705">
-        <v>3520</v>
+        <v>1053</v>
       </c>
       <c r="C705" t="s">
-        <v>876</v>
+        <v>1265</v>
       </c>
     </row>
     <row r="706" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A706" t="s">
-        <v>872</v>
+        <v>1262</v>
       </c>
       <c r="B706">
-        <v>764</v>
+        <v>1086</v>
       </c>
       <c r="C706" t="s">
-        <v>876</v>
+        <v>1265</v>
       </c>
     </row>
     <row r="707" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A707" t="s">
-        <v>873</v>
+        <v>1263</v>
       </c>
       <c r="B707">
-        <v>2035</v>
+        <v>5574</v>
       </c>
       <c r="C707" t="s">
-        <v>876</v>
+        <v>1265</v>
       </c>
     </row>
     <row r="708" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A708" t="s">
-        <v>874</v>
+        <v>1264</v>
       </c>
       <c r="B708">
-        <v>900</v>
+        <v>892</v>
       </c>
       <c r="C708" t="s">
-        <v>876</v>
+        <v>1265</v>
       </c>
     </row>
     <row r="709" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A709" t="s">
-        <v>875</v>
+        <v>1265</v>
       </c>
       <c r="B709">
-        <v>1172</v>
+        <v>952</v>
       </c>
       <c r="C709" t="s">
-        <v>876</v>
+        <v>1265</v>
       </c>
     </row>
     <row r="710" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A710" t="s">
-        <v>876</v>
+        <v>1266</v>
       </c>
       <c r="B710">
-        <v>962</v>
+        <v>3575</v>
       </c>
       <c r="C710" t="s">
-        <v>876</v>
+        <v>1265</v>
       </c>
     </row>
     <row r="711" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A711" t="s">
-        <v>877</v>
+        <v>1267</v>
       </c>
       <c r="B711">
-        <v>2494</v>
+        <v>1018</v>
       </c>
       <c r="C711" t="s">
-        <v>876</v>
+        <v>1265</v>
       </c>
     </row>
     <row r="712" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A712" t="s">
-        <v>878</v>
+        <v>1560</v>
       </c>
       <c r="B712">
-        <v>8025</v>
+        <v>8026</v>
       </c>
       <c r="C712" t="s">
         <v>876</v>
@@ -31238,10 +31268,10 @@
     </row>
     <row r="713" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A713" t="s">
-        <v>879</v>
+        <v>870</v>
       </c>
       <c r="B713">
-        <v>1015</v>
+        <v>2495</v>
       </c>
       <c r="C713" t="s">
         <v>876</v>
@@ -31249,274 +31279,274 @@
     </row>
     <row r="714" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A714" t="s">
-        <v>1268</v>
+        <v>871</v>
       </c>
       <c r="B714">
-        <v>310</v>
+        <v>3520</v>
       </c>
       <c r="C714" t="s">
-        <v>1274</v>
+        <v>876</v>
       </c>
     </row>
     <row r="715" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A715" t="s">
-        <v>1269</v>
+        <v>872</v>
       </c>
       <c r="B715">
-        <v>321</v>
+        <v>764</v>
       </c>
       <c r="C715" t="s">
-        <v>1274</v>
+        <v>876</v>
       </c>
     </row>
     <row r="716" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A716" t="s">
-        <v>1270</v>
+        <v>873</v>
       </c>
       <c r="B716">
-        <v>306</v>
+        <v>2035</v>
       </c>
       <c r="C716" t="s">
-        <v>1274</v>
+        <v>876</v>
       </c>
     </row>
     <row r="717" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A717" t="s">
-        <v>1271</v>
+        <v>874</v>
       </c>
       <c r="B717">
-        <v>322</v>
+        <v>900</v>
       </c>
       <c r="C717" t="s">
-        <v>1274</v>
+        <v>876</v>
       </c>
     </row>
     <row r="718" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A718" t="s">
-        <v>1272</v>
+        <v>875</v>
       </c>
       <c r="B718">
-        <v>311</v>
+        <v>1172</v>
       </c>
       <c r="C718" t="s">
-        <v>1274</v>
+        <v>876</v>
       </c>
     </row>
     <row r="719" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A719" t="s">
-        <v>1273</v>
+        <v>876</v>
       </c>
       <c r="B719">
-        <v>2798</v>
+        <v>962</v>
       </c>
       <c r="C719" t="s">
-        <v>1274</v>
+        <v>876</v>
       </c>
     </row>
     <row r="720" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A720" t="s">
-        <v>1274</v>
+        <v>877</v>
       </c>
       <c r="B720">
-        <v>12</v>
+        <v>2494</v>
       </c>
       <c r="C720" t="s">
-        <v>1274</v>
+        <v>876</v>
       </c>
     </row>
     <row r="721" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A721" t="s">
-        <v>1275</v>
+        <v>878</v>
       </c>
       <c r="B721">
-        <v>2797</v>
+        <v>8025</v>
       </c>
       <c r="C721" t="s">
-        <v>1274</v>
+        <v>876</v>
       </c>
     </row>
     <row r="722" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A722" t="s">
-        <v>1620</v>
+        <v>879</v>
       </c>
       <c r="B722">
-        <v>3977</v>
+        <v>1015</v>
       </c>
       <c r="C722" t="s">
-        <v>1276</v>
+        <v>876</v>
       </c>
     </row>
     <row r="723" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A723" t="s">
-        <v>1276</v>
+        <v>1268</v>
       </c>
       <c r="B723">
-        <v>1998</v>
+        <v>310</v>
       </c>
       <c r="C723" t="s">
-        <v>1276</v>
+        <v>1274</v>
       </c>
     </row>
     <row r="724" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A724" t="s">
-        <v>1277</v>
+        <v>1269</v>
       </c>
       <c r="B724">
-        <v>5905</v>
+        <v>321</v>
       </c>
       <c r="C724" t="s">
-        <v>1278</v>
+        <v>1274</v>
       </c>
     </row>
     <row r="725" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A725" t="s">
-        <v>1278</v>
+        <v>1270</v>
       </c>
       <c r="B725">
-        <v>973</v>
+        <v>306</v>
       </c>
       <c r="C725" t="s">
-        <v>1278</v>
+        <v>1274</v>
       </c>
     </row>
     <row r="726" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A726" t="s">
-        <v>880</v>
+        <v>1271</v>
       </c>
       <c r="B726">
-        <v>6570</v>
+        <v>322</v>
       </c>
       <c r="C726" t="s">
-        <v>881</v>
+        <v>1274</v>
       </c>
     </row>
     <row r="727" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A727" t="s">
-        <v>881</v>
-      </c>
-      <c r="B727" t="e">
-        <v>#N/A</v>
+        <v>1272</v>
+      </c>
+      <c r="B727">
+        <v>311</v>
       </c>
       <c r="C727" t="s">
-        <v>881</v>
+        <v>1274</v>
       </c>
     </row>
     <row r="728" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A728" t="s">
-        <v>882</v>
-      </c>
-      <c r="B728" t="e">
-        <v>#N/A</v>
+        <v>1273</v>
+      </c>
+      <c r="B728">
+        <v>2798</v>
       </c>
       <c r="C728" t="s">
-        <v>881</v>
+        <v>1274</v>
       </c>
     </row>
     <row r="729" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A729" t="s">
-        <v>1279</v>
+        <v>1274</v>
       </c>
       <c r="B729">
-        <v>31</v>
+        <v>12</v>
       </c>
       <c r="C729" t="s">
-        <v>1290</v>
+        <v>1274</v>
       </c>
     </row>
     <row r="730" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A730" t="s">
-        <v>1280</v>
+        <v>1275</v>
       </c>
       <c r="B730">
-        <v>52</v>
+        <v>2797</v>
       </c>
       <c r="C730" t="s">
-        <v>1290</v>
+        <v>1274</v>
       </c>
     </row>
     <row r="731" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A731" t="s">
-        <v>1281</v>
+        <v>1620</v>
       </c>
       <c r="B731">
-        <v>51</v>
+        <v>3977</v>
       </c>
       <c r="C731" t="s">
-        <v>1290</v>
+        <v>1276</v>
       </c>
     </row>
     <row r="732" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A732" t="s">
-        <v>1282</v>
+        <v>1276</v>
       </c>
       <c r="B732">
-        <v>1157</v>
+        <v>1998</v>
       </c>
       <c r="C732" t="s">
-        <v>1290</v>
+        <v>1276</v>
       </c>
     </row>
     <row r="733" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A733" t="s">
-        <v>1283</v>
+        <v>1277</v>
       </c>
       <c r="B733">
-        <v>2187</v>
+        <v>5905</v>
       </c>
       <c r="C733" t="s">
-        <v>1290</v>
+        <v>1278</v>
       </c>
     </row>
     <row r="734" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A734" t="s">
-        <v>1284</v>
+        <v>1278</v>
       </c>
       <c r="B734">
-        <v>50</v>
+        <v>973</v>
       </c>
       <c r="C734" t="s">
-        <v>1290</v>
+        <v>1278</v>
       </c>
     </row>
     <row r="735" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A735" t="s">
-        <v>1285</v>
+        <v>880</v>
       </c>
       <c r="B735">
-        <v>33</v>
+        <v>6570</v>
       </c>
       <c r="C735" t="s">
-        <v>1290</v>
+        <v>881</v>
       </c>
     </row>
     <row r="736" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A736" t="s">
-        <v>1286</v>
+        <v>881</v>
       </c>
       <c r="B736">
-        <v>4225</v>
+        <v>3267</v>
       </c>
       <c r="C736" t="s">
-        <v>1290</v>
+        <v>881</v>
       </c>
     </row>
     <row r="737" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A737" t="s">
-        <v>1287</v>
+        <v>882</v>
       </c>
       <c r="B737">
-        <v>177</v>
+        <v>986</v>
       </c>
       <c r="C737" t="s">
-        <v>1290</v>
+        <v>881</v>
       </c>
     </row>
     <row r="738" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A738" t="s">
-        <v>1288</v>
+        <v>1279</v>
       </c>
       <c r="B738">
-        <v>1156</v>
+        <v>31</v>
       </c>
       <c r="C738" t="s">
         <v>1290</v>
@@ -31524,10 +31554,10 @@
     </row>
     <row r="739" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A739" t="s">
-        <v>897</v>
+        <v>1280</v>
       </c>
       <c r="B739">
-        <v>45</v>
+        <v>52</v>
       </c>
       <c r="C739" t="s">
         <v>1290</v>
@@ -31535,10 +31565,10 @@
     </row>
     <row r="740" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A740" t="s">
-        <v>1289</v>
+        <v>1281</v>
       </c>
       <c r="B740">
-        <v>2</v>
+        <v>51</v>
       </c>
       <c r="C740" t="s">
         <v>1290</v>
@@ -31546,10 +31576,10 @@
     </row>
     <row r="741" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A741" t="s">
-        <v>1290</v>
+        <v>1282</v>
       </c>
       <c r="B741">
-        <v>1</v>
+        <v>1157</v>
       </c>
       <c r="C741" t="s">
         <v>1290</v>
@@ -31557,10 +31587,10 @@
     </row>
     <row r="742" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A742" t="s">
-        <v>1291</v>
+        <v>1283</v>
       </c>
       <c r="B742">
-        <v>46</v>
+        <v>2187</v>
       </c>
       <c r="C742" t="s">
         <v>1290</v>
@@ -31568,10 +31598,10 @@
     </row>
     <row r="743" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A743" t="s">
-        <v>1292</v>
+        <v>1284</v>
       </c>
       <c r="B743">
-        <v>3578</v>
+        <v>50</v>
       </c>
       <c r="C743" t="s">
         <v>1290</v>
@@ -31579,142 +31609,142 @@
     </row>
     <row r="744" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A744" t="s">
-        <v>1293</v>
+        <v>1285</v>
       </c>
       <c r="B744">
-        <v>2598</v>
+        <v>33</v>
       </c>
       <c r="C744" t="s">
-        <v>1295</v>
+        <v>1290</v>
       </c>
     </row>
     <row r="745" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A745" t="s">
-        <v>1294</v>
+        <v>1286</v>
       </c>
       <c r="B745">
-        <v>3792</v>
+        <v>4225</v>
       </c>
       <c r="C745" t="s">
-        <v>1295</v>
+        <v>1290</v>
       </c>
     </row>
     <row r="746" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A746" t="s">
-        <v>1295</v>
+        <v>1287</v>
       </c>
       <c r="B746">
-        <v>1938</v>
+        <v>177</v>
       </c>
       <c r="C746" t="s">
-        <v>1295</v>
+        <v>1290</v>
       </c>
     </row>
     <row r="747" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A747" t="s">
-        <v>1621</v>
+        <v>1288</v>
       </c>
       <c r="B747">
-        <v>6584</v>
+        <v>1156</v>
       </c>
       <c r="C747" t="s">
-        <v>1300</v>
+        <v>1290</v>
       </c>
     </row>
     <row r="748" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A748" t="s">
-        <v>1296</v>
+        <v>897</v>
       </c>
       <c r="B748">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="C748" t="s">
-        <v>1300</v>
+        <v>1290</v>
       </c>
     </row>
     <row r="749" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A749" t="s">
-        <v>1297</v>
+        <v>1289</v>
       </c>
       <c r="B749">
-        <v>40</v>
+        <v>2</v>
       </c>
       <c r="C749" t="s">
-        <v>1300</v>
+        <v>1290</v>
       </c>
     </row>
     <row r="750" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A750" t="s">
-        <v>1622</v>
+        <v>1290</v>
       </c>
       <c r="B750">
-        <v>6586</v>
+        <v>1</v>
       </c>
       <c r="C750" t="s">
-        <v>1300</v>
+        <v>1290</v>
       </c>
     </row>
     <row r="751" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A751" t="s">
-        <v>1298</v>
+        <v>1291</v>
       </c>
       <c r="B751">
-        <v>3412</v>
+        <v>46</v>
       </c>
       <c r="C751" t="s">
-        <v>1300</v>
+        <v>1290</v>
       </c>
     </row>
     <row r="752" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A752" t="s">
-        <v>1623</v>
+        <v>1292</v>
       </c>
       <c r="B752">
-        <v>6587</v>
+        <v>3578</v>
       </c>
       <c r="C752" t="s">
-        <v>1300</v>
+        <v>1290</v>
       </c>
     </row>
     <row r="753" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A753" t="s">
-        <v>1624</v>
+        <v>1293</v>
       </c>
       <c r="B753">
-        <v>6585</v>
+        <v>2598</v>
       </c>
       <c r="C753" t="s">
-        <v>1300</v>
+        <v>1295</v>
       </c>
     </row>
     <row r="754" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A754" t="s">
-        <v>1625</v>
+        <v>1294</v>
       </c>
       <c r="B754">
-        <v>39</v>
+        <v>3792</v>
       </c>
       <c r="C754" t="s">
-        <v>1300</v>
+        <v>1295</v>
       </c>
     </row>
     <row r="755" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A755" t="s">
-        <v>1299</v>
+        <v>1295</v>
       </c>
       <c r="B755">
-        <v>38</v>
+        <v>1938</v>
       </c>
       <c r="C755" t="s">
-        <v>1300</v>
+        <v>1295</v>
       </c>
     </row>
     <row r="756" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A756" t="s">
-        <v>1626</v>
+        <v>1621</v>
       </c>
       <c r="B756">
-        <v>41</v>
+        <v>6584</v>
       </c>
       <c r="C756" t="s">
         <v>1300</v>
@@ -31722,10 +31752,10 @@
     </row>
     <row r="757" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A757" t="s">
-        <v>1300</v>
+        <v>1296</v>
       </c>
       <c r="B757">
-        <v>37</v>
+        <v>44</v>
       </c>
       <c r="C757" t="s">
         <v>1300</v>
@@ -31733,10 +31763,10 @@
     </row>
     <row r="758" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A758" t="s">
-        <v>1627</v>
+        <v>1297</v>
       </c>
       <c r="B758">
-        <v>6583</v>
+        <v>40</v>
       </c>
       <c r="C758" t="s">
         <v>1300</v>
@@ -31744,109 +31774,109 @@
     </row>
     <row r="759" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A759" t="s">
-        <v>1301</v>
+        <v>1622</v>
       </c>
       <c r="B759">
-        <v>403</v>
+        <v>6586</v>
       </c>
       <c r="C759" t="s">
-        <v>1630</v>
+        <v>1300</v>
       </c>
     </row>
     <row r="760" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A760" t="s">
-        <v>1302</v>
+        <v>1298</v>
       </c>
       <c r="B760">
-        <v>4720</v>
+        <v>3412</v>
       </c>
       <c r="C760" t="s">
-        <v>1630</v>
+        <v>1300</v>
       </c>
     </row>
     <row r="761" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A761" t="s">
-        <v>705</v>
+        <v>1623</v>
       </c>
       <c r="B761">
-        <v>16</v>
+        <v>6587</v>
       </c>
       <c r="C761" t="s">
-        <v>1630</v>
+        <v>1300</v>
       </c>
     </row>
     <row r="762" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A762" t="s">
-        <v>1303</v>
+        <v>1624</v>
       </c>
       <c r="B762">
-        <v>4721</v>
+        <v>6585</v>
       </c>
       <c r="C762" t="s">
-        <v>1630</v>
+        <v>1300</v>
       </c>
     </row>
     <row r="763" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A763" t="s">
-        <v>1304</v>
+        <v>1625</v>
       </c>
       <c r="B763">
-        <v>462</v>
+        <v>39</v>
       </c>
       <c r="C763" t="s">
-        <v>1630</v>
+        <v>1300</v>
       </c>
     </row>
     <row r="764" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A764" t="s">
-        <v>1628</v>
+        <v>1299</v>
       </c>
       <c r="B764">
-        <v>399</v>
+        <v>38</v>
       </c>
       <c r="C764" t="s">
-        <v>1630</v>
+        <v>1300</v>
       </c>
     </row>
     <row r="765" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A765" t="s">
-        <v>1305</v>
+        <v>1626</v>
       </c>
       <c r="B765">
-        <v>4726</v>
+        <v>41</v>
       </c>
       <c r="C765" t="s">
-        <v>1630</v>
+        <v>1300</v>
       </c>
     </row>
     <row r="766" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A766" t="s">
-        <v>1306</v>
+        <v>1300</v>
       </c>
       <c r="B766">
-        <v>6049</v>
+        <v>37</v>
       </c>
       <c r="C766" t="s">
-        <v>1630</v>
+        <v>1300</v>
       </c>
     </row>
     <row r="767" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A767" t="s">
-        <v>1307</v>
+        <v>1627</v>
       </c>
       <c r="B767">
-        <v>4731</v>
+        <v>6583</v>
       </c>
       <c r="C767" t="s">
-        <v>1630</v>
+        <v>1300</v>
       </c>
     </row>
     <row r="768" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A768" t="s">
-        <v>1308</v>
+        <v>1301</v>
       </c>
       <c r="B768">
-        <v>4744</v>
+        <v>403</v>
       </c>
       <c r="C768" t="s">
         <v>1630</v>
@@ -31854,10 +31884,10 @@
     </row>
     <row r="769" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A769" t="s">
-        <v>1309</v>
+        <v>1302</v>
       </c>
       <c r="B769">
-        <v>4748</v>
+        <v>4720</v>
       </c>
       <c r="C769" t="s">
         <v>1630</v>
@@ -31865,10 +31895,10 @@
     </row>
     <row r="770" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A770" t="s">
-        <v>1310</v>
+        <v>705</v>
       </c>
       <c r="B770">
-        <v>468</v>
+        <v>16</v>
       </c>
       <c r="C770" t="s">
         <v>1630</v>
@@ -31876,10 +31906,10 @@
     </row>
     <row r="771" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A771" t="s">
-        <v>1311</v>
+        <v>1303</v>
       </c>
       <c r="B771">
-        <v>401</v>
+        <v>4721</v>
       </c>
       <c r="C771" t="s">
         <v>1630</v>
@@ -31887,10 +31917,10 @@
     </row>
     <row r="772" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A772" t="s">
-        <v>1312</v>
+        <v>1304</v>
       </c>
       <c r="B772">
-        <v>15</v>
+        <v>462</v>
       </c>
       <c r="C772" t="s">
         <v>1630</v>
@@ -31898,18 +31928,117 @@
     </row>
     <row r="773" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A773" t="s">
-        <v>1313</v>
+        <v>1628</v>
       </c>
       <c r="B773">
-        <v>6050</v>
+        <v>399</v>
       </c>
       <c r="C773" t="s">
         <v>1630</v>
       </c>
     </row>
+    <row r="774" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A774" t="s">
+        <v>1305</v>
+      </c>
+      <c r="B774">
+        <v>4726</v>
+      </c>
+      <c r="C774" t="s">
+        <v>1630</v>
+      </c>
+    </row>
+    <row r="775" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A775" t="s">
+        <v>1306</v>
+      </c>
+      <c r="B775">
+        <v>6049</v>
+      </c>
+      <c r="C775" t="s">
+        <v>1630</v>
+      </c>
+    </row>
+    <row r="776" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A776" t="s">
+        <v>1307</v>
+      </c>
+      <c r="B776">
+        <v>4731</v>
+      </c>
+      <c r="C776" t="s">
+        <v>1630</v>
+      </c>
+    </row>
+    <row r="777" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A777" t="s">
+        <v>1308</v>
+      </c>
+      <c r="B777">
+        <v>4744</v>
+      </c>
+      <c r="C777" t="s">
+        <v>1630</v>
+      </c>
+    </row>
+    <row r="778" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A778" t="s">
+        <v>1309</v>
+      </c>
+      <c r="B778">
+        <v>4748</v>
+      </c>
+      <c r="C778" t="s">
+        <v>1630</v>
+      </c>
+    </row>
+    <row r="779" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A779" t="s">
+        <v>1310</v>
+      </c>
+      <c r="B779">
+        <v>468</v>
+      </c>
+      <c r="C779" t="s">
+        <v>1630</v>
+      </c>
+    </row>
+    <row r="780" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A780" t="s">
+        <v>1311</v>
+      </c>
+      <c r="B780">
+        <v>401</v>
+      </c>
+      <c r="C780" t="s">
+        <v>1630</v>
+      </c>
+    </row>
+    <row r="781" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A781" t="s">
+        <v>1312</v>
+      </c>
+      <c r="B781">
+        <v>15</v>
+      </c>
+      <c r="C781" t="s">
+        <v>1630</v>
+      </c>
+    </row>
+    <row r="782" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A782" t="s">
+        <v>1313</v>
+      </c>
+      <c r="B782">
+        <v>6050</v>
+      </c>
+      <c r="C782" t="s">
+        <v>1630</v>
+      </c>
+    </row>
   </sheetData>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:C773">
-    <sortCondition ref="C2:C773"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:C782">
+    <sortCondition ref="C2:C782"/>
   </sortState>
   <conditionalFormatting sqref="B1:B1048576">
     <cfRule type="duplicateValues" dxfId="0" priority="1"/>

</xml_diff>